<commit_message>
Update ZK01-ZK09 quotation pricing
</commit_message>
<xml_diff>
--- a/assets/files/quotes/ZK05-quotation.xlsx
+++ b/assets/files/quotes/ZK05-quotation.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English Quotation" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'中文报价单'!$A$11:$E$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'English Quotation'!$A$11:$E$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'中文报价单'!$A$11:$E$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'English Quotation'!$A$11:$E$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -631,9 +631,11 @@
       <c r="E5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="6" t="n"/>
+      <c r="A6" s="6" t="n">
+        <v>620000</v>
+      </c>
       <c r="B6" s="6">
-        <f>IF(SUM(D12:D40)=0,"",SUM(D12:D40))</f>
+        <f>IF(SUM(D12:D44)=0,"",SUM(D12:D44))</f>
         <v/>
       </c>
       <c r="C6" s="6">
@@ -679,12 +681,14 @@
           <t>ZK05 露台舱</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
+      <c r="B9" s="9" t="n">
+        <v>620000</v>
+      </c>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>项目定制</t>
+          <t>露台、户外休闲、景区度假基础配置</t>
         </is>
       </c>
     </row>
@@ -725,11 +729,11 @@
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>全套卫浴 / 带洗浴</t>
+          <t>露台户外休闲包</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>25000</v>
+        <v>85000</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
@@ -740,16 +744,20 @@
         <f>IF($C12="☑",$B12,"")</f>
         <v/>
       </c>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>户外露台、休闲座椅、遮阳及景观布置</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>储物柜（衣物收纳）</t>
+          <t>活动运营移动部署包</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>7000</v>
+        <v>120000</v>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
@@ -760,16 +768,20 @@
         <f>IF($C13="☑",$B13,"")</f>
         <v/>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>牵引、支撑腿、户外接口及快速转场结构</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>床及床垫（单套）</t>
+          <t>户外遮阳棚 / 雨棚</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>9300</v>
+        <v>28000</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
@@ -780,16 +792,20 @@
         <f>IF($C14="☑",$B14,"")</f>
         <v/>
       </c>
-      <c r="E14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>适合露台、营地和景区休闲区</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>第二床位 / 第二床垫</t>
+          <t>户外家具与景观灯</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>3200</v>
+        <v>22000</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
@@ -800,16 +816,20 @@
         <f>IF($C15="☑",$B15,"")</f>
         <v/>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>露台桌椅、氛围灯和景观照明</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>桌椅套装</t>
+          <t>全套卫浴 / 带洗浴</t>
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>2500</v>
+        <v>25000</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
@@ -825,11 +845,11 @@
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>电器包</t>
+          <t>储物柜（衣物收纳）</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>40000</v>
+        <v>7000</v>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
@@ -845,11 +865,11 @@
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>电动窗帘</t>
+          <t>床及床垫（单套）</t>
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>5700</v>
+        <v>9300</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
@@ -865,11 +885,11 @@
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Low-E 玻璃升级</t>
+          <t>第二床位 / 第二床垫</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>20000</v>
+        <v>3200</v>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
@@ -885,11 +905,11 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>天窗</t>
+          <t>桌椅套装</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>15000</v>
+        <v>2500</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
@@ -905,7 +925,7 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>内饰升级包</t>
+          <t>电器包</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
@@ -925,11 +945,11 @@
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>地暖系统</t>
+          <t>电动窗帘</t>
         </is>
       </c>
       <c r="B22" s="10" t="n">
-        <v>20000</v>
+        <v>5700</v>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
@@ -945,11 +965,11 @@
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>灯带 / 氛围照明系统</t>
+          <t>Low-E 玻璃升级</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
@@ -965,11 +985,11 @@
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>中央空调</t>
+          <t>天窗</t>
         </is>
       </c>
       <c r="B24" s="10" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
@@ -985,11 +1005,11 @@
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>挂机空调</t>
+          <t>内饰升级包</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>4700</v>
+        <v>40000</v>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
@@ -1005,11 +1025,11 @@
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>新风系统</t>
+          <t>地暖系统</t>
         </is>
       </c>
       <c r="B26" s="10" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
@@ -1025,11 +1045,11 @@
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>顶部太阳能光伏板</t>
+          <t>灯带 / 氛围照明系统</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>25000</v>
+        <v>2500</v>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
@@ -1045,11 +1065,11 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>储能电池系统</t>
+          <t>中央空调</t>
         </is>
       </c>
       <c r="B28" s="10" t="n">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
@@ -1065,11 +1085,11 @@
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>逆变器 / 能源管理系统</t>
+          <t>挂机空调</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>20000</v>
+        <v>4700</v>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
@@ -1085,11 +1105,11 @@
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>星链连接硬件及安装辅材</t>
+          <t>新风系统</t>
         </is>
       </c>
       <c r="B30" s="10" t="n">
-        <v>33200</v>
+        <v>15000</v>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
@@ -1105,11 +1125,11 @@
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>国际通信系统</t>
+          <t>顶部太阳能光伏板</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>10800</v>
+        <v>25000</v>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
@@ -1125,11 +1145,11 @@
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>LED 大屏幕</t>
+          <t>储能电池系统</t>
         </is>
       </c>
       <c r="B32" s="10" t="n">
-        <v>28000</v>
+        <v>50000</v>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
@@ -1145,11 +1165,11 @@
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>投影仪</t>
+          <t>逆变器 / 能源管理系统</t>
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>5800</v>
+        <v>20000</v>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
@@ -1165,11 +1185,11 @@
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>3D 展示系统</t>
+          <t>星链连接硬件及安装辅材</t>
         </is>
       </c>
       <c r="B34" s="10" t="n">
-        <v>25000</v>
+        <v>33200</v>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
@@ -1185,11 +1205,11 @@
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AI 智能全系统</t>
+          <t>国际通信系统</t>
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>100000</v>
+        <v>10800</v>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
@@ -1205,11 +1225,11 @@
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>AI 语音控制 / 设备联动全屋智能</t>
+          <t>LED 大屏幕</t>
         </is>
       </c>
       <c r="B36" s="10" t="n">
-        <v>20000</v>
+        <v>28000</v>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
@@ -1225,11 +1245,11 @@
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>净水系统</t>
+          <t>投影仪</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
-        <v>10000</v>
+        <v>5800</v>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
@@ -1245,11 +1265,11 @@
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>智能门锁</t>
+          <t>3D 展示系统</t>
         </is>
       </c>
       <c r="B38" s="10" t="n">
-        <v>1600</v>
+        <v>25000</v>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
@@ -1265,11 +1285,11 @@
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>监控 / 烟感 / 水浸报警基础包</t>
+          <t>AI 智能全系统</t>
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>4700</v>
+        <v>100000</v>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
@@ -1285,11 +1305,11 @@
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>运输成本合计</t>
+          <t>AI 语音控制 / 设备联动全屋智能</t>
         </is>
       </c>
       <c r="B40" s="10" t="n">
-        <v>96700</v>
+        <v>20000</v>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
@@ -1302,18 +1322,98 @@
       </c>
       <c r="E40" s="4" t="inlineStr"/>
     </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>净水系统</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D41" s="9">
+        <f>IF($C41="☑",$B41,"")</f>
+        <v/>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>智能门锁</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D42" s="10">
+        <f>IF($C42="☑",$B42,"")</f>
+        <v/>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>监控 / 烟感 / 水浸报警基础包</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>4700</v>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D43" s="9">
+        <f>IF($C43="☑",$B43,"")</f>
+        <v/>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>运输成本合计</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>96700</v>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D44" s="10">
+        <f>IF($C44="☑",$B44,"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A11:E40"/>
+  <autoFilter ref="A11:E44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A12:E40">
+  <conditionalFormatting sqref="A12:E44">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$C12="☑"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C12:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid value" error="Please select from the list" promptTitle="Checkbox" prompt="Select checkbox" type="list">
+    <dataValidation sqref="C12:C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid value" error="Please select from the list" promptTitle="Checkbox" prompt="Select checkbox" type="list">
       <formula1>"☐,☑"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1328,7 +1428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1426,9 +1526,11 @@
       <c r="E5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="6" t="n"/>
+      <c r="A6" s="6" t="n">
+        <v>620000</v>
+      </c>
       <c r="B6" s="6">
-        <f>IF(SUM(D12:D40)=0,"",SUM(D12:D40))</f>
+        <f>IF(SUM(D12:D44)=0,"",SUM(D12:D44))</f>
         <v/>
       </c>
       <c r="C6" s="6">
@@ -1474,12 +1576,14 @@
           <t>ZK05 Terrace Capsule</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
+      <c r="B9" s="9" t="n">
+        <v>620000</v>
+      </c>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Customized project</t>
+          <t>Terrace, outdoor leisure and resort-use base configuration</t>
         </is>
       </c>
     </row>
@@ -1520,11 +1624,11 @@
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Complete bathroom / shower</t>
+          <t>Terrace outdoor leisure package</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>25000</v>
+        <v>85000</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
@@ -1535,16 +1639,20 @@
         <f>IF($C12="☑",$B12,"")</f>
         <v/>
       </c>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Outdoor terrace, leisure seating, shading and landscape setup</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Storage cabinet / wardrobe</t>
+          <t>Mobile deployment package for events</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>7000</v>
+        <v>120000</v>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
@@ -1555,16 +1663,20 @@
         <f>IF($C13="☑",$B13,"")</f>
         <v/>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Towing, support legs, outdoor interfaces and quick relocation structure</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Bed and mattress set</t>
+          <t>Outdoor canopy / awning</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>9300</v>
+        <v>28000</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
@@ -1575,16 +1687,20 @@
         <f>IF($C14="☑",$B14,"")</f>
         <v/>
       </c>
-      <c r="E14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Suitable for terraces, campsites and resort leisure areas</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Second bed / second mattress</t>
+          <t>Outdoor furniture and landscape lighting</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>3200</v>
+        <v>22000</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
@@ -1595,16 +1711,20 @@
         <f>IF($C15="☑",$B15,"")</f>
         <v/>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Terrace furniture, ambient lighting and landscape lights</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Desk and chair set</t>
+          <t>Complete bathroom / shower</t>
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>2500</v>
+        <v>25000</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
@@ -1620,11 +1740,11 @@
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Appliance package</t>
+          <t>Storage cabinet / wardrobe</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>40000</v>
+        <v>7000</v>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
@@ -1640,11 +1760,11 @@
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Motorized curtains</t>
+          <t>Bed and mattress set</t>
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>5700</v>
+        <v>9300</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
@@ -1660,11 +1780,11 @@
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Low-E glass upgrade</t>
+          <t>Second bed / second mattress</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>20000</v>
+        <v>3200</v>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
@@ -1680,11 +1800,11 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Skylight</t>
+          <t>Desk and chair set</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>15000</v>
+        <v>2500</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
@@ -1700,7 +1820,7 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Interior finish upgrade package</t>
+          <t>Appliance package</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
@@ -1720,11 +1840,11 @@
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Floor heating system</t>
+          <t>Motorized curtains</t>
         </is>
       </c>
       <c r="B22" s="10" t="n">
-        <v>20000</v>
+        <v>5700</v>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
@@ -1740,11 +1860,11 @@
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Light strip / ambient lighting system</t>
+          <t>Low-E glass upgrade</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
@@ -1760,11 +1880,11 @@
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Central air conditioning</t>
+          <t>Skylight</t>
         </is>
       </c>
       <c r="B24" s="10" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
@@ -1780,11 +1900,11 @@
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Wall-mounted air conditioner</t>
+          <t>Interior finish upgrade package</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>4700</v>
+        <v>40000</v>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
@@ -1800,11 +1920,11 @@
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Fresh air ventilation system</t>
+          <t>Floor heating system</t>
         </is>
       </c>
       <c r="B26" s="10" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
@@ -1820,11 +1940,11 @@
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Roof solar PV panels</t>
+          <t>Light strip / ambient lighting system</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>25000</v>
+        <v>2500</v>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
@@ -1840,11 +1960,11 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Energy storage battery system</t>
+          <t>Central air conditioning</t>
         </is>
       </c>
       <c r="B28" s="10" t="n">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
@@ -1860,11 +1980,11 @@
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Inverter / energy management system</t>
+          <t>Wall-mounted air conditioner</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>20000</v>
+        <v>4700</v>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
@@ -1880,11 +2000,11 @@
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Starlink hardware and installation accessories</t>
+          <t>Fresh air ventilation system</t>
         </is>
       </c>
       <c r="B30" s="10" t="n">
-        <v>33200</v>
+        <v>15000</v>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
@@ -1900,11 +2020,11 @@
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>International communication system</t>
+          <t>Roof solar PV panels</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>10800</v>
+        <v>25000</v>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
@@ -1920,11 +2040,11 @@
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>LED display screen</t>
+          <t>Energy storage battery system</t>
         </is>
       </c>
       <c r="B32" s="10" t="n">
-        <v>28000</v>
+        <v>50000</v>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
@@ -1940,11 +2060,11 @@
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Projector</t>
+          <t>Inverter / energy management system</t>
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>5800</v>
+        <v>20000</v>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
@@ -1960,11 +2080,11 @@
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>3D presentation system</t>
+          <t>Starlink hardware and installation accessories</t>
         </is>
       </c>
       <c r="B34" s="10" t="n">
-        <v>25000</v>
+        <v>33200</v>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
@@ -1980,11 +2100,11 @@
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AI smart system</t>
+          <t>International communication system</t>
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>100000</v>
+        <v>10800</v>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
@@ -2000,11 +2120,11 @@
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>AI voice control / device-linked smart system</t>
+          <t>LED display screen</t>
         </is>
       </c>
       <c r="B36" s="10" t="n">
-        <v>20000</v>
+        <v>28000</v>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
@@ -2020,11 +2140,11 @@
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Water purification system</t>
+          <t>Projector</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
-        <v>10000</v>
+        <v>5800</v>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
@@ -2040,11 +2160,11 @@
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Smart door lock</t>
+          <t>3D presentation system</t>
         </is>
       </c>
       <c r="B38" s="10" t="n">
-        <v>1600</v>
+        <v>25000</v>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
@@ -2060,11 +2180,11 @@
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Basic security package</t>
+          <t>AI smart system</t>
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>4700</v>
+        <v>100000</v>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
@@ -2080,11 +2200,11 @@
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Estimated logistics cost</t>
+          <t>AI voice control / device-linked smart system</t>
         </is>
       </c>
       <c r="B40" s="10" t="n">
-        <v>96700</v>
+        <v>20000</v>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
@@ -2097,18 +2217,98 @@
       </c>
       <c r="E40" s="4" t="inlineStr"/>
     </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Water purification system</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D41" s="9">
+        <f>IF($C41="☑",$B41,"")</f>
+        <v/>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Smart door lock</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D42" s="10">
+        <f>IF($C42="☑",$B42,"")</f>
+        <v/>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Basic security package</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>4700</v>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D43" s="9">
+        <f>IF($C43="☑",$B43,"")</f>
+        <v/>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Estimated logistics cost</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>96700</v>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="D44" s="10">
+        <f>IF($C44="☑",$B44,"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A11:E40"/>
+  <autoFilter ref="A11:E44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A12:E40">
+  <conditionalFormatting sqref="A12:E44">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$C12="☑"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C12:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid value" error="Please select from the list" promptTitle="Checkbox" prompt="Select checkbox" type="list">
+    <dataValidation sqref="C12:C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid value" error="Please select from the list" promptTitle="Checkbox" prompt="Select checkbox" type="list">
       <formula1>"☐,☑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>